<commit_message>
change(reporting): use previous close as reference price, not next-session open
Reporting layer only — screener and evaluator.py unchanged. Reference price is
now the PREVIOUS CLOSE (close of the signal session); the next valid session's
High/Close are measured against it:
  %High  = (High  - Prev)/Prev*100
  %Close = (Close - Prev)/Prev*100
  W/L    = W if Close > Prev
Columns are now: Signal, Prev, Close, High, %High, %Close, W/L (CSV + Excel +
dashboard). Pending/backfill behaviour preserved (no faked values). Daily CSV/
Excel and signal_results.csv regenerated with the new schema.

Verified on real data: 2026-06-08 swing 5W/2L (WR 71.4%), scalping 4W/8L
(33.3%); e.g. FORU.JK prev 2020 (06-08 close) → 06-09 close 2460 = +21.78% W.
</commit_message>
<xml_diff>
--- a/data/performance/daily/signal_list_2026-05-07.xlsx
+++ b/data/performance/daily/signal_list_2026-05-07.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">

</xml_diff>